<commit_message>
with bug fixes for calc_pir and wired in wnvSurv
</commit_message>
<xml_diff>
--- a/3_output/2026/w29/y2026_w29_weekly_report_output.xlsx
+++ b/3_output/2026/w29/y2026_w29_weekly_report_output.xlsx
@@ -3238,7 +3238,7 @@
         <v>56</v>
       </c>
       <c r="D23" s="26" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="E23" s="26" t="s">
         <v>56</v>
@@ -3262,7 +3262,7 @@
         <v>56</v>
       </c>
       <c r="L23" s="26" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="M23" s="26" t="s">
         <v>56</v>
@@ -3376,13 +3376,13 @@
         <v>56</v>
       </c>
       <c r="H25" s="26" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="I25" s="16" t="s">
         <v>56</v>
       </c>
       <c r="J25" s="26" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="K25" s="16" t="s">
         <v>56</v>
@@ -3553,7 +3553,7 @@
         <v>58</v>
       </c>
       <c r="D28" s="26" t="n">
-        <v>0.18</v>
+        <v>0.21</v>
       </c>
       <c r="E28" s="16" t="s">
         <v>58</v>
@@ -3577,7 +3577,7 @@
         <v>58</v>
       </c>
       <c r="L28" s="26" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="M28" s="16" t="s">
         <v>58</v>
@@ -3679,7 +3679,7 @@
         <v>58</v>
       </c>
       <c r="D30" s="26" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="E30" s="16" t="s">
         <v>58</v>
@@ -3691,7 +3691,7 @@
         <v>58</v>
       </c>
       <c r="H30" s="26" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="I30" s="16" t="s">
         <v>58</v>
@@ -3742,13 +3742,13 @@
         <v>58</v>
       </c>
       <c r="D31" s="26" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="E31" s="16" t="s">
         <v>58</v>
       </c>
       <c r="F31" s="26" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="G31" s="16" t="s">
         <v>58</v>
@@ -3805,7 +3805,7 @@
         <v>58</v>
       </c>
       <c r="D32" s="26" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E32" s="16" t="s">
         <v>58</v>
@@ -3823,13 +3823,13 @@
         <v>58</v>
       </c>
       <c r="J32" s="26" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="K32" s="16" t="s">
         <v>58</v>
       </c>
       <c r="L32" s="26" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="M32" s="16" t="s">
         <v>58</v>
@@ -3886,7 +3886,7 @@
         <v>58</v>
       </c>
       <c r="J33" s="26" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K33" s="16" t="s">
         <v>58</v>
@@ -3931,7 +3931,7 @@
         <v>58</v>
       </c>
       <c r="D34" s="26" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="E34" s="16" t="s">
         <v>58</v>
@@ -6887,7 +6887,7 @@
         <v>56</v>
       </c>
       <c r="D90" s="14" t="n">
-        <v>3.3</v>
+        <v>6</v>
       </c>
       <c r="E90" s="14" t="s">
         <v>56</v>
@@ -6911,7 +6911,7 @@
         <v>56</v>
       </c>
       <c r="L90" s="14" t="n">
-        <v>0.5</v>
+        <v>0.72</v>
       </c>
       <c r="M90" s="14" t="s">
         <v>56</v>
@@ -7025,19 +7025,19 @@
         <v>56</v>
       </c>
       <c r="H92" s="14" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="I92" s="14" t="s">
         <v>56</v>
       </c>
       <c r="J92" s="14" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="K92" s="14" t="s">
         <v>56</v>
       </c>
       <c r="L92" s="14" t="n">
-        <v>1.52</v>
+        <v>1.54</v>
       </c>
       <c r="M92" s="16" t="s">
         <v>56</v>
@@ -7100,7 +7100,7 @@
         <v>56</v>
       </c>
       <c r="L93" s="14" t="n">
-        <v>3.42</v>
+        <v>3.4</v>
       </c>
       <c r="M93" s="16" t="s">
         <v>56</v>
@@ -7202,7 +7202,7 @@
         <v>58</v>
       </c>
       <c r="D95" s="14" t="n">
-        <v>5.66</v>
+        <v>6.34</v>
       </c>
       <c r="E95" s="14" t="s">
         <v>58</v>
@@ -7226,7 +7226,7 @@
         <v>58</v>
       </c>
       <c r="L95" s="14" t="n">
-        <v>5.52</v>
+        <v>5.6</v>
       </c>
       <c r="M95" s="16" t="s">
         <v>58</v>
@@ -7265,31 +7265,31 @@
         <v>58</v>
       </c>
       <c r="D96" s="14" t="n">
-        <v>10.48</v>
+        <v>10.46</v>
       </c>
       <c r="E96" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F96" s="14" t="n">
-        <v>5.66</v>
+        <v>5.64</v>
       </c>
       <c r="G96" s="14" t="s">
         <v>58</v>
       </c>
       <c r="H96" s="14" t="n">
-        <v>8.52</v>
+        <v>8.5</v>
       </c>
       <c r="I96" s="14" t="s">
         <v>58</v>
       </c>
       <c r="J96" s="14" t="n">
-        <v>10.38</v>
+        <v>10.34</v>
       </c>
       <c r="K96" s="14" t="s">
         <v>58</v>
       </c>
       <c r="L96" s="14" t="n">
-        <v>7.86</v>
+        <v>7.84</v>
       </c>
       <c r="M96" s="16" t="s">
         <v>58</v>
@@ -7328,31 +7328,31 @@
         <v>58</v>
       </c>
       <c r="D97" s="14" t="n">
-        <v>10.98</v>
+        <v>10.84</v>
       </c>
       <c r="E97" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F97" s="14" t="n">
-        <v>8.44</v>
+        <v>8.4</v>
       </c>
       <c r="G97" s="14" t="s">
         <v>58</v>
       </c>
       <c r="H97" s="14" t="n">
-        <v>8.74</v>
+        <v>8.68</v>
       </c>
       <c r="I97" s="14" t="s">
         <v>58</v>
       </c>
       <c r="J97" s="14" t="n">
-        <v>12.16</v>
+        <v>12.12</v>
       </c>
       <c r="K97" s="14" t="s">
         <v>58</v>
       </c>
       <c r="L97" s="14" t="n">
-        <v>10.82</v>
+        <v>10.76</v>
       </c>
       <c r="M97" s="16" t="s">
         <v>58</v>
@@ -7391,31 +7391,31 @@
         <v>58</v>
       </c>
       <c r="D98" s="14" t="n">
-        <v>12.16</v>
+        <v>12.74</v>
       </c>
       <c r="E98" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F98" s="14" t="n">
-        <v>12.56</v>
+        <v>13.3</v>
       </c>
       <c r="G98" s="14" t="s">
         <v>58</v>
       </c>
       <c r="H98" s="14" t="n">
-        <v>9.18</v>
+        <v>9.16</v>
       </c>
       <c r="I98" s="14" t="s">
         <v>58</v>
       </c>
       <c r="J98" s="14" t="n">
-        <v>17.74</v>
+        <v>17.48</v>
       </c>
       <c r="K98" s="14" t="s">
         <v>58</v>
       </c>
       <c r="L98" s="14" t="n">
-        <v>11.74</v>
+        <v>11.94</v>
       </c>
       <c r="M98" s="16" t="s">
         <v>58</v>
@@ -7454,31 +7454,31 @@
         <v>58</v>
       </c>
       <c r="D99" s="14" t="n">
-        <v>4.14</v>
+        <v>5.02</v>
       </c>
       <c r="E99" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F99" s="14" t="n">
-        <v>8.62</v>
+        <v>8.58</v>
       </c>
       <c r="G99" s="14" t="s">
         <v>58</v>
       </c>
       <c r="H99" s="14" t="n">
-        <v>12.44</v>
+        <v>12.08</v>
       </c>
       <c r="I99" s="14" t="s">
         <v>58</v>
       </c>
       <c r="J99" s="14" t="n">
-        <v>13.16</v>
+        <v>15</v>
       </c>
       <c r="K99" s="14" t="s">
         <v>58</v>
       </c>
       <c r="L99" s="14" t="n">
-        <v>8.3</v>
+        <v>8.7</v>
       </c>
       <c r="M99" s="16" t="s">
         <v>58</v>
@@ -7517,7 +7517,7 @@
         <v>58</v>
       </c>
       <c r="D100" s="14" t="n">
-        <v>17.74</v>
+        <v>17.08</v>
       </c>
       <c r="E100" s="14" t="s">
         <v>58</v>
@@ -7529,19 +7529,19 @@
         <v>58</v>
       </c>
       <c r="H100" s="14" t="n">
-        <v>10.06</v>
+        <v>9.92</v>
       </c>
       <c r="I100" s="14" t="s">
         <v>58</v>
       </c>
       <c r="J100" s="14" t="n">
-        <v>4.96</v>
+        <v>8.16</v>
       </c>
       <c r="K100" s="14" t="s">
         <v>58</v>
       </c>
       <c r="L100" s="14" t="n">
-        <v>7.12</v>
+        <v>7.42</v>
       </c>
       <c r="M100" s="16" t="s">
         <v>58</v>
@@ -7580,31 +7580,31 @@
         <v>58</v>
       </c>
       <c r="D101" s="14" t="n">
-        <v>7.24</v>
+        <v>6.7</v>
       </c>
       <c r="E101" s="14" t="s">
         <v>58</v>
       </c>
       <c r="F101" s="14" t="n">
-        <v>4.38</v>
+        <v>4.34</v>
       </c>
       <c r="G101" s="14" t="s">
         <v>58</v>
       </c>
       <c r="H101" s="14" t="n">
-        <v>3.44</v>
+        <v>3.32</v>
       </c>
       <c r="I101" s="14" t="s">
         <v>58</v>
       </c>
       <c r="J101" s="14" t="n">
-        <v>5.94</v>
+        <v>5.22</v>
       </c>
       <c r="K101" s="14" t="s">
         <v>58</v>
       </c>
       <c r="L101" s="14" t="n">
-        <v>5.04</v>
+        <v>4.84</v>
       </c>
       <c r="M101" s="16" t="s">
         <v>58</v>
@@ -46075,7 +46075,7 @@
         <v>56</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="D5" t="s">
         <v>56</v>
@@ -46099,7 +46099,7 @@
         <v>56</v>
       </c>
       <c r="K5" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="L5" t="s">
         <v>56</v>
@@ -46175,13 +46175,13 @@
         <v>56</v>
       </c>
       <c r="G7" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="H7" t="s">
         <v>56</v>
       </c>
       <c r="I7" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="J7" t="s">
         <v>56</v>
@@ -46295,7 +46295,7 @@
         <v>58</v>
       </c>
       <c r="C10" t="n">
-        <v>0.18</v>
+        <v>0.21</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
@@ -46319,7 +46319,7 @@
         <v>58</v>
       </c>
       <c r="K10" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="L10" t="s">
         <v>58</v>
@@ -46383,7 +46383,7 @@
         <v>58</v>
       </c>
       <c r="C12" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="D12" t="s">
         <v>58</v>
@@ -46395,7 +46395,7 @@
         <v>58</v>
       </c>
       <c r="G12" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="H12" t="s">
         <v>58</v>
@@ -46427,13 +46427,13 @@
         <v>58</v>
       </c>
       <c r="C13" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="D13" t="s">
         <v>58</v>
       </c>
       <c r="E13" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="F13" t="s">
         <v>58</v>
@@ -46471,7 +46471,7 @@
         <v>58</v>
       </c>
       <c r="C14" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="D14" t="s">
         <v>58</v>
@@ -46489,13 +46489,13 @@
         <v>58</v>
       </c>
       <c r="I14" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="J14" t="s">
         <v>58</v>
       </c>
       <c r="K14" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="L14" t="s">
         <v>58</v>
@@ -46533,7 +46533,7 @@
         <v>58</v>
       </c>
       <c r="I15" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="J15" t="s">
         <v>58</v>
@@ -46559,7 +46559,7 @@
         <v>58</v>
       </c>
       <c r="C16" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="D16" t="s">
         <v>58</v>
@@ -48143,7 +48143,7 @@
         <v>56</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
         <v>56</v>
@@ -48167,7 +48167,7 @@
         <v>56</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5</v>
+        <v>0.72</v>
       </c>
       <c r="L5" t="s">
         <v>56</v>
@@ -48243,19 +48243,19 @@
         <v>56</v>
       </c>
       <c r="G7" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="H7" t="s">
         <v>56</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="J7" t="s">
         <v>56</v>
       </c>
       <c r="K7" t="n">
-        <v>1.52</v>
+        <v>1.54</v>
       </c>
       <c r="L7" t="s">
         <v>56</v>
@@ -48299,7 +48299,7 @@
         <v>56</v>
       </c>
       <c r="K8" t="n">
-        <v>3.42</v>
+        <v>3.4</v>
       </c>
       <c r="L8" t="s">
         <v>56</v>
@@ -48363,7 +48363,7 @@
         <v>58</v>
       </c>
       <c r="C10" t="n">
-        <v>5.66</v>
+        <v>6.34</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
@@ -48387,7 +48387,7 @@
         <v>58</v>
       </c>
       <c r="K10" t="n">
-        <v>5.52</v>
+        <v>5.6</v>
       </c>
       <c r="L10" t="s">
         <v>58</v>
@@ -48407,31 +48407,31 @@
         <v>58</v>
       </c>
       <c r="C11" t="n">
-        <v>10.48</v>
+        <v>10.46</v>
       </c>
       <c r="D11" t="s">
         <v>58</v>
       </c>
       <c r="E11" t="n">
-        <v>5.66</v>
+        <v>5.64</v>
       </c>
       <c r="F11" t="s">
         <v>58</v>
       </c>
       <c r="G11" t="n">
-        <v>8.52</v>
+        <v>8.5</v>
       </c>
       <c r="H11" t="s">
         <v>58</v>
       </c>
       <c r="I11" t="n">
-        <v>10.38</v>
+        <v>10.34</v>
       </c>
       <c r="J11" t="s">
         <v>58</v>
       </c>
       <c r="K11" t="n">
-        <v>7.86</v>
+        <v>7.84</v>
       </c>
       <c r="L11" t="s">
         <v>58</v>
@@ -48451,31 +48451,31 @@
         <v>58</v>
       </c>
       <c r="C12" t="n">
-        <v>10.98</v>
+        <v>10.84</v>
       </c>
       <c r="D12" t="s">
         <v>58</v>
       </c>
       <c r="E12" t="n">
-        <v>8.44</v>
+        <v>8.4</v>
       </c>
       <c r="F12" t="s">
         <v>58</v>
       </c>
       <c r="G12" t="n">
-        <v>8.74</v>
+        <v>8.68</v>
       </c>
       <c r="H12" t="s">
         <v>58</v>
       </c>
       <c r="I12" t="n">
-        <v>12.16</v>
+        <v>12.12</v>
       </c>
       <c r="J12" t="s">
         <v>58</v>
       </c>
       <c r="K12" t="n">
-        <v>10.82</v>
+        <v>10.76</v>
       </c>
       <c r="L12" t="s">
         <v>58</v>
@@ -48495,31 +48495,31 @@
         <v>58</v>
       </c>
       <c r="C13" t="n">
-        <v>12.16</v>
+        <v>12.74</v>
       </c>
       <c r="D13" t="s">
         <v>58</v>
       </c>
       <c r="E13" t="n">
-        <v>12.56</v>
+        <v>13.3</v>
       </c>
       <c r="F13" t="s">
         <v>58</v>
       </c>
       <c r="G13" t="n">
-        <v>9.18</v>
+        <v>9.16</v>
       </c>
       <c r="H13" t="s">
         <v>58</v>
       </c>
       <c r="I13" t="n">
-        <v>17.74</v>
+        <v>17.48</v>
       </c>
       <c r="J13" t="s">
         <v>58</v>
       </c>
       <c r="K13" t="n">
-        <v>11.74</v>
+        <v>11.94</v>
       </c>
       <c r="L13" t="s">
         <v>58</v>
@@ -48539,31 +48539,31 @@
         <v>58</v>
       </c>
       <c r="C14" t="n">
-        <v>4.14</v>
+        <v>5.02</v>
       </c>
       <c r="D14" t="s">
         <v>58</v>
       </c>
       <c r="E14" t="n">
-        <v>8.62</v>
+        <v>8.58</v>
       </c>
       <c r="F14" t="s">
         <v>58</v>
       </c>
       <c r="G14" t="n">
-        <v>12.44</v>
+        <v>12.08</v>
       </c>
       <c r="H14" t="s">
         <v>58</v>
       </c>
       <c r="I14" t="n">
-        <v>13.16</v>
+        <v>15</v>
       </c>
       <c r="J14" t="s">
         <v>58</v>
       </c>
       <c r="K14" t="n">
-        <v>8.3</v>
+        <v>8.7</v>
       </c>
       <c r="L14" t="s">
         <v>58</v>
@@ -48583,7 +48583,7 @@
         <v>58</v>
       </c>
       <c r="C15" t="n">
-        <v>17.74</v>
+        <v>17.08</v>
       </c>
       <c r="D15" t="s">
         <v>58</v>
@@ -48595,19 +48595,19 @@
         <v>58</v>
       </c>
       <c r="G15" t="n">
-        <v>10.06</v>
+        <v>9.92</v>
       </c>
       <c r="H15" t="s">
         <v>58</v>
       </c>
       <c r="I15" t="n">
-        <v>4.96</v>
+        <v>8.16</v>
       </c>
       <c r="J15" t="s">
         <v>58</v>
       </c>
       <c r="K15" t="n">
-        <v>7.12</v>
+        <v>7.42</v>
       </c>
       <c r="L15" t="s">
         <v>58</v>
@@ -48627,31 +48627,31 @@
         <v>58</v>
       </c>
       <c r="C16" t="n">
-        <v>7.24</v>
+        <v>6.7</v>
       </c>
       <c r="D16" t="s">
         <v>58</v>
       </c>
       <c r="E16" t="n">
-        <v>4.38</v>
+        <v>4.34</v>
       </c>
       <c r="F16" t="s">
         <v>58</v>
       </c>
       <c r="G16" t="n">
-        <v>3.44</v>
+        <v>3.32</v>
       </c>
       <c r="H16" t="s">
         <v>58</v>
       </c>
       <c r="I16" t="n">
-        <v>5.94</v>
+        <v>5.22</v>
       </c>
       <c r="J16" t="s">
         <v>58</v>
       </c>
       <c r="K16" t="n">
-        <v>5.04</v>
+        <v>4.84</v>
       </c>
       <c r="L16" t="s">
         <v>58</v>

</xml_diff>